<commit_message>
add machine image auto-prediction (romaji matching) + master
- 機種画像紐づけページに自動予測（pykakasiローマ字化）を追加
- machine_image_master.xlsx を更新
- requirements に pykakasi 追加

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/masters/machine_image_master.xlsx
+++ b/masters/machine_image_master.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -464,6 +464,1350 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>BIRDIE WING</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>birdiewing</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GALFY</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>galfy</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>HEY鏡</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>kagami</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>LBマジハロ</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>LBmajiharo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>LB不二子</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>fujiko</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Lドラハナ閃光</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>drahanasenko</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Lハナビ</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>lhanabi</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>L攻殻機動隊</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>koukaku</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>L沖ドキDUO</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>okidokiduo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>L絶対衝激</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>zettaishogeki4</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Newクレア</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>kurea</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SAO</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>sao</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>SBJ</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>sbj</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ToLOVEる</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>toloveru</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>うみねこ2</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>umineko2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>かぐや様</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>kaguya</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>からくりサーカス</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>karakuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>このすば</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>konosuba</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>わた婚</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>watakon</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>アクダマドライブ</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>akudama</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>アズールレーン</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>azuren</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>アニスロドッチ</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>anislodotch</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ウルトラミラジャグ</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ultramirajug</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>エウレカART</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>eurekaart</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>エリサラ鏡</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>kagami</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>キンハナ30</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>kinghanahana30</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>クレアの秘宝伝</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>hihouden</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>グランベルム</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>guranberumu</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>ゴッド神々の軌跡</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>godkamigami</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>シャーマンキング</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>shamanking</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>スマスロドラハナ閃光</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>drahanasenko</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>スマスロ化物語</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>bakemonogatari</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>スマスロ北斗の拳</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>hokuto</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>スマスロ秘宝伝</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>hihouden</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>スマートキンハナV</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>smartkinhanav</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>スーパーBJ</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>sbj</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>タクトオーパス</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>taktop</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ダリフラ</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>darifra</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ダークハイビ</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>darkhaibi</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>チバリヨ2</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>chibariyo2</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>ディスクアップUR</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>diskupur</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>ドラハナ閃光30</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>drahanasenko</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>ネオアイム</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>neoim</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>バイオ5</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>vio5</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>バイオRE:3</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>biore3</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>バジ絆2天膳</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>basitenzen</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>プリズムナナ</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>prismnana</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>マギレコ</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>magireko</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>マクロスF4</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>macrossf4</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>マクロスデルタ</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>macrossdelta</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>マジハロToT</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>LBmajiharo</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>モンハンライズ</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>monhunrise</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>ユニコーン覚醒</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>unicornkakusei</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>ヨルムンガンド</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>yorumungando</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>リオエース2</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>rioace2</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ヱヴァ約束</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>evayakusoku</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>主役は銭形5</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>zenigata5</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>吉宗</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>yoshimune</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>戦国乙女4</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>sengokuotome4</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>戦国乙女5</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>sengokuotome5</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>新ハナビ</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>shinhanabi</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>新鬼武者3</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>shinoni3</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>沖ドキBLACK</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>okidokiblack</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>沖ドキGOLD</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>okidokigold</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>沖ドキGOLD30</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>okidokigold30</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>沖ドキゴージャス30</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>okidokigorgeous30</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>異世界かるてっと</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>isekai</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>真打吉宗</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>shinuchiyoshimune</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>範馬刃牙</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>hanmabaki</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>絶対衝激IV</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>zettaishogeki4</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>虚構推理</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>kyokousuiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>鉄拳6</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>tekken6</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>銀河英雄伝説</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>gingaeiyu</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>いざ!番長</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>izabantyo</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>アレックスB</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>arex</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>LBサンダーV</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>lbthunderv</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>LBシェイク</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>shake</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>LBトリプルクラウン</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>triplecrown</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>SAOII</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>sao2</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ToLOVEるトランス</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>toloveru87</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>とある超電磁砲2</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>toaru2</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>カバネリ海門決戦</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>kabaneriunato</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>クランキークレスト</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>cranky</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>ゴッドイーター</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>godeater</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>ゴブスレII</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>goblinslayer2</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>ゴージャグ3</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>gojug</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>シンフォギア正義</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>symphogear</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ジャグラーガールズ</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>jugglergirls</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>スタァライト</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>starlight</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ディスクアップ2</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>discup2</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>ドルアーガの塔</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>druaga</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>ネオプラ</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>neoplanet</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>ハピジャグV</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>happyjug</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>バーサスリヴァイズ</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>versusrexse</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>バーニングEXP.</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>burning</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>ビッグドリーム</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>bigdream</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>ファンキー2</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>funkyjug</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>ホウオウ天翔30</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>hanahanahouoh30</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>マイジャグV</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>myjug5</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>マジハロ8</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>magimallo8</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>ミスジャグ</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>mrjuggler</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>モンキーターンV</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>monkey5</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>ヴァルヴレイヴ2</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>vvv2</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>北斗転生2</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>hokutotensei2</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>東京リベンジャーズ</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>tokyorevengers</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>東京喰種</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>tokyoghoul</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>炎炎ノ消防隊2</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>enen2</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>無職転生</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>musyoku</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>聖闘士星矢</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>seiya</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>転剣</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>tenken</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>防振り</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>boufuri</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>キンハナV30</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>kinhana30</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>